<commit_message>
Added import items form excel file
</commit_message>
<xml_diff>
--- a/Sample Data/ITEMS-SAMPLE.xlsx
+++ b/Sample Data/ITEMS-SAMPLE.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30417"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="57" documentId="11_39E067654ADF7ED3EA39FA7889A3541B62FF829C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{90AF8EF1-34AC-4985-9208-26B128F8DDB9}"/>
+  <xr:revisionPtr revIDLastSave="60" documentId="11_39E067654ADF7ED3EA39FA7889A3541B62FF829C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7F6D301F-0A14-42CF-B62A-CAC11E7ECADD}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="25">
   <si>
     <t>PART NO</t>
   </si>
@@ -106,6 +106,9 @@
   </si>
   <si>
     <t>07000-15310</t>
+  </si>
+  <si>
+    <t>2W8003</t>
   </si>
 </sst>
 </file>
@@ -458,7 +461,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
@@ -576,6 +579,17 @@
         <v>22</v>
       </c>
     </row>
+    <row r="11" spans="1:3">
+      <c r="A11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>